<commit_message>
reducing wait time from 5s to 2s
</commit_message>
<xml_diff>
--- a/SampleTestKitsWithData/Testkit_HTTP_1/TC01_Start/environment.xlsx
+++ b/SampleTestKitsWithData/Testkit_HTTP_1/TC01_Start/environment.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3EEA631-B854-4855-A177-3DD6030F9026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14292F07-1999-4989-916A-EC042D6F702B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
     <sheet name="Action" sheetId="3" r:id="rId2"/>
     <sheet name="FileType" sheetId="4" state="hidden" r:id="rId3"/>
     <sheet name="ElementType" sheetId="5" state="hidden" r:id="rId4"/>
-    <sheet name="Run" sheetId="6" r:id="rId8"/>
+    <sheet name="Run" sheetId="6" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191028" fullCalcOnLoad="1" fullPrecision="1"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="47">
   <si>
     <t>Key</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Default_Database_Name</t>
   </si>
   <si>
-    <t>database</t>
-  </si>
-  <si>
     <t>Default_Database_File_Path</t>
   </si>
   <si>
@@ -165,18 +162,20 @@
   </si>
   <si>
     <t>reset_database</t>
+  </si>
+  <si>
+    <t>Library</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -196,7 +195,7 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -361,75 +360,75 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="2" applyFill="1" borderId="1" applyBorder="1" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="2" applyFill="1" borderId="1" applyBorder="1" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" applyFill="1" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="2" applyFill="1" borderId="2" applyBorder="1" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="2" applyFill="1" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="2" applyFill="1" borderId="3" applyBorder="1" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" applyFont="1" fillId="3" applyFill="1" borderId="4" applyBorder="1" xfId="0"/>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="0" borderId="4" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="0" borderId="4" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="4" applyFill="1" borderId="4" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="4" applyFill="1" borderId="4" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" applyFill="1" borderId="4" applyBorder="1" xfId="0"/>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="2" applyFill="1" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="2" applyFill="1" borderId="2" applyBorder="1" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="2" applyFill="1" borderId="3" applyBorder="1" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" applyFont="1" fillId="5" applyFill="1" borderId="5" applyBorder="1" xfId="0"/>
-    <xf numFmtId="0" fontId="6" applyFont="1" fillId="5" applyFill="1" borderId="6" applyBorder="1" xfId="0"/>
-    <xf numFmtId="0" fontId="7" applyFont="1" fillId="0" borderId="7" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" applyFont="1" fillId="0" borderId="8" applyBorder="1" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,18 +436,30 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border>
         <left style="thin">
-          <color rgb="ff000000"/>
+          <color rgb="FF000000"/>
         </left>
-        <right style="thin">
-          <color rgb="ff000000"/>
-        </right>
         <top style="thin">
-          <color rgb="ff000000"/>
+          <color rgb="FF000000"/>
         </top>
         <bottom style="thin">
-          <color rgb="ff000000"/>
+          <color rgb="FF000000"/>
         </bottom>
       </border>
     </dxf>
@@ -463,45 +474,33 @@
         <shadow val="0"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color rgb="ff000000"/>
+        <color rgb="FF000000"/>
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border>
         <top style="thin">
-          <color rgb="ff000000"/>
+          <color rgb="FF000000"/>
         </top>
         <bottom style="thin">
-          <color rgb="ff000000"/>
+          <color rgb="FF000000"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="ff000000"/>
-        <name val="Calibri"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border>
         <left style="thin">
-          <color rgb="ff000000"/>
+          <color rgb="FF000000"/>
         </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
         <top style="thin">
-          <color rgb="ff000000"/>
+          <color rgb="FF000000"/>
         </top>
         <bottom style="thin">
-          <color rgb="ff000000"/>
+          <color rgb="FF000000"/>
         </bottom>
       </border>
     </dxf>
@@ -519,11 +518,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{054913B0-5323-4F83-856A-AA921BB86A96}" name="Table1" displayName="Table1" ref="A1:B2" totalsRowShown="0" tableBorderDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{054913B0-5323-4F83-856A-AA921BB86A96}" name="Table1" displayName="Table1" ref="A1:B2" totalsRowShown="0" tableBorderDxfId="2">
   <autoFilter ref="A1:B2" xr:uid="{054913B0-5323-4F83-856A-AA921BB86A96}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{EEF80A4C-AE1A-42E1-8D02-233D6645FC7A}" name="Step" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{1E0B1333-A75D-493C-BE3E-968ECB29CDD7}" name="Keyword action" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{1E0B1333-A75D-493C-BE3E-968ECB29CDD7}" name="Keyword action" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -793,13 +792,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="1" width="27.6328125" customWidth="1"/>
-    <col min="2" max="2" width="43.6328125" customWidth="1"/>
+    <col min="1" max="1" width="27.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -807,7 +806,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>2</v>
       </c>
@@ -815,317 +814,317 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="0" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="s">
+      <c r="B5" s="18" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A77F7F08-67CF-4D6B-8968-79F94E5D3D47}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.6328125" customWidth="1" style="11"/>
-    <col min="2" max="2" width="37.1796875" customWidth="1" style="12"/>
+    <col min="1" max="1" width="21.59765625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="37.19921875" style="12" customWidth="1"/>
     <col min="3" max="3" width="66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="23" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="19" t="s">
+      <c r="B2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="9" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="23"/>
+      <c r="B3" s="9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="19"/>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="9" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="23"/>
+      <c r="B4" s="9" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="19"/>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="9" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="23"/>
+      <c r="B5" s="9" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19"/>
-      <c r="B5" s="9" t="s">
+      <c r="C5" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="9" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="23"/>
+      <c r="B6" s="9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="19"/>
-      <c r="B6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="10" t="s">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="24" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="20" t="s">
+      <c r="B7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="C7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="9" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="23"/>
+      <c r="B8" s="9" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="19"/>
-      <c r="B8" s="9" t="s">
+      <c r="C8" s="9"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="23"/>
+      <c r="B9" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="9"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="19"/>
-      <c r="B9" s="9" t="s">
+      <c r="C9" s="9"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="23"/>
+      <c r="B10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="9"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="19"/>
-      <c r="B10" s="9" t="s">
+      <c r="C10" s="9"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="25"/>
+      <c r="B11" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="9"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="21"/>
-      <c r="B11" s="10" t="s">
-        <v>30</v>
-      </c>
       <c r="C11" s="10"/>
     </row>
   </sheetData>
-  <mergeCells>
+  <mergeCells count="2">
     <mergeCell ref="A2:A6"/>
     <mergeCell ref="A7:A11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{360E1C82-158F-43FD-AAE3-57AC0D969288}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="17.1796875" customWidth="1"/>
-    <col min="3" max="3" width="15.6328125" customWidth="1"/>
+    <col min="2" max="2" width="17.19921875" customWidth="1"/>
+    <col min="3" max="3" width="15.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="s">
-        <v>35</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4973CF49-F632-40AC-AD8F-E0F1A942FCB5}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.08984375" customWidth="1"/>
-    <col min="2" max="2" width="24.08984375" customWidth="1"/>
+    <col min="1" max="1" width="20.09765625" customWidth="1"/>
+    <col min="2" max="2" width="24.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" s="4"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
       <c r="B5" s="6"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="6"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C078E10-675F-4787-89DC-8EE857A7C94A}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" customWidth="1"/>
-    <col min="2" max="2" width="36.109375" customWidth="1"/>
+    <col min="1" max="1" width="7.296875" customWidth="1"/>
+    <col min="2" max="2" width="36.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="23" t="s">
+    </row>
+    <row r="2" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="21">
+        <v>1</v>
+      </c>
+      <c r="B2" s="22" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="24">
-        <v>1</v>
-      </c>
-      <c r="B2" s="25" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
         <v>46</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>